<commit_message>
Auto commit at 2026-05-21  9:33:01.62
</commit_message>
<xml_diff>
--- a/data/hzsj.xlsx
+++ b/data/hzsj.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="171">
   <si>
     <t>充电时间</t>
   </si>
@@ -1013,7 +1013,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N440"/>
+  <dimension ref="A1:N438"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.75" style="5" bestFit="1" customWidth="1"/>
@@ -3824,50 +3824,22 @@
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A117" s="9">
-        <v>46023</v>
-      </c>
-      <c r="B117" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C117" s="1">
-        <v>419557.75</v>
-      </c>
-      <c r="D117" s="1">
-        <v>196768.98</v>
-      </c>
-      <c r="E117" s="1">
-        <v>120867.02</v>
-      </c>
-      <c r="F117" s="1">
-        <v>317636</v>
-      </c>
-      <c r="G117" s="1">
-        <v>17783</v>
-      </c>
+      <c r="A117" s="4"/>
+      <c r="B117" s="4"/>
+      <c r="C117" s="1"/>
+      <c r="D117" s="1"/>
+      <c r="E117" s="1"/>
+      <c r="F117" s="1"/>
+      <c r="G117" s="1"/>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A118" s="9">
-        <v>46023</v>
-      </c>
-      <c r="B118" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C118" s="1">
-        <v>160938.26999999999</v>
-      </c>
-      <c r="D118" s="1">
-        <v>91508.68</v>
-      </c>
-      <c r="E118" s="1">
-        <v>43542.5</v>
-      </c>
-      <c r="F118" s="1">
-        <v>135051.18</v>
-      </c>
-      <c r="G118" s="1">
-        <v>5690</v>
-      </c>
+      <c r="A118" s="4"/>
+      <c r="B118" s="4"/>
+      <c r="C118" s="1"/>
+      <c r="D118" s="1"/>
+      <c r="E118" s="1"/>
+      <c r="F118" s="1"/>
+      <c r="G118" s="1"/>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.15">
       <c r="A119" s="4"/>
@@ -6748,24 +6720,6 @@
       <c r="E438" s="1"/>
       <c r="F438" s="1"/>
       <c r="G438" s="1"/>
-    </row>
-    <row r="439" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A439" s="4"/>
-      <c r="B439" s="4"/>
-      <c r="C439" s="1"/>
-      <c r="D439" s="1"/>
-      <c r="E439" s="1"/>
-      <c r="F439" s="1"/>
-      <c r="G439" s="1"/>
-    </row>
-    <row r="440" spans="1:7" x14ac:dyDescent="0.15">
-      <c r="A440" s="4"/>
-      <c r="B440" s="4"/>
-      <c r="C440" s="1"/>
-      <c r="D440" s="1"/>
-      <c r="E440" s="1"/>
-      <c r="F440" s="1"/>
-      <c r="G440" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>